<commit_message>
Use "short" error codes for config files
</commit_message>
<xml_diff>
--- a/src/PhpSpreadsheet/Calculation/locale/Translations.xlsx
+++ b/src/PhpSpreadsheet/Calculation/locale/Translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\PHPOffice\PHPSpreadsheet\develop\src\PhpSpreadsheet\Calculation\locale\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFC82EE7-E78E-43E5-86E0-F7C6B93F2BA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22B96276-825E-4349-AF5A-109120426D20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4406" yWindow="1243" windowWidth="24685" windowHeight="16723" tabRatio="989" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8604" uniqueCount="6511">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8611" uniqueCount="6515">
   <si>
     <t>SUBTOTAL</t>
   </si>
@@ -19602,6 +19602,18 @@
   </si>
   <si>
     <t>Slovenščina</t>
+  </si>
+  <si>
+    <t>NULL</t>
+  </si>
+  <si>
+    <t>REF</t>
+  </si>
+  <si>
+    <t>NAME</t>
+  </si>
+  <si>
+    <t>DIV0</t>
   </si>
 </sst>
 </file>
@@ -20353,9 +20365,11 @@
       </c>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.4">
-      <c r="A8" s="2"/>
+      <c r="A8" s="3" t="s">
+        <v>6344</v>
+      </c>
       <c r="B8" s="3" t="s">
-        <v>6344</v>
+        <v>6511</v>
       </c>
       <c r="C8" t="s">
         <v>6352</v>
@@ -20416,8 +20430,11 @@
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.4">
+      <c r="A9" s="3" t="s">
+        <v>6471</v>
+      </c>
       <c r="B9" s="3" t="s">
-        <v>6471</v>
+        <v>6514</v>
       </c>
       <c r="C9" t="s">
         <v>6366</v>
@@ -20463,8 +20480,11 @@
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.4">
+      <c r="A10" s="3" t="s">
+        <v>6472</v>
+      </c>
       <c r="B10" s="3" t="s">
-        <v>6472</v>
+        <v>748</v>
       </c>
       <c r="C10" t="s">
         <v>6380</v>
@@ -20543,8 +20563,11 @@
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.4">
+      <c r="A11" s="3" t="s">
+        <v>6473</v>
+      </c>
       <c r="B11" s="3" t="s">
-        <v>6473</v>
+        <v>6512</v>
       </c>
       <c r="C11" t="s">
         <v>6403</v>
@@ -20596,8 +20619,11 @@
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.4">
+      <c r="A12" s="3" t="s">
+        <v>6474</v>
+      </c>
       <c r="B12" s="3" t="s">
-        <v>6474</v>
+        <v>6513</v>
       </c>
       <c r="C12" t="s">
         <v>6418</v>
@@ -20673,8 +20699,11 @@
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.4">
+      <c r="A13" s="3" t="s">
+        <v>6475</v>
+      </c>
       <c r="B13" s="3" t="s">
-        <v>6475</v>
+        <v>3070</v>
       </c>
       <c r="C13" t="s">
         <v>6437</v>
@@ -20735,8 +20764,11 @@
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.4">
+      <c r="A14" s="3" t="s">
+        <v>6476</v>
+      </c>
       <c r="B14" s="3" t="s">
-        <v>6476</v>
+        <v>300</v>
       </c>
       <c r="C14" t="s">
         <v>6453</v>

</xml_diff>